<commit_message>
fix(verification): GW3 carries the vendor's conductivity
gw003's k was the builder's 1e-5 default; the vendor model's own SK is
1e-7 m/s. The problem is confined and homogeneous, so the published
head-profile targets do not move (re-measured: all five within
0.011 m of the chart values, tag green), and the self-locked flowrate
scales exactly with k: 2.351e-05 -> 2.351e-07, updated as an explicit
pair. Figure regenerated, 29/29 rebuild, page recertified. Also on
SEEP-4: the phreatic paragraph now answers the drain-pressure question
directly — an active exit face is held at atmospheric, all thirteen
nodes stay active, so the drain runs at zero pressure head end to end
and the zero-pressure line past x = 40 is the drain itself.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjjT2aBxw8gY7EFdpoUcpj
</commit_message>
<xml_diff>
--- a/docs/verification/files/rocscience_gw/gw003.xlsx
+++ b/docs/verification/files/rocscience_gw/gw003.xlsx
@@ -6650,10 +6650,10 @@
         <v>0.0</v>
       </c>
       <c r="AG11" s="3">
-        <v>1e-05</v>
+        <v>1e-07</v>
       </c>
       <c r="AH11" s="3">
-        <v>1e-05</v>
+        <v>1e-07</v>
       </c>
       <c r="AI11" s="3">
         <v>0.0</v>

</xml_diff>